<commit_message>
docs: update case study documents and add new prioritization guide for AI use cases
This commit includes significant updates to existing case study documents and introduces a new markdown file focused on prioritizing AI use cases. Key changes include:

1. **G01_Enterprise_Knowledge_Assistant.md**: Updated to reflect changes in section contributions and clarify the design and implementation details.
2. **New File: 60_Prioritize_AI_Use_Cases.md**: A comprehensive guide outlining a structured approach to prioritizing AI use cases in large enterprises, including criteria for selection and evaluation.

These updates aim to enhance the interview preparation materials by providing clearer insights and actionable strategies for AI implementation.
</commit_message>
<xml_diff>
--- a/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
+++ b/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
@@ -200,9 +200,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseStudies" displayName="CaseStudies" ref="A1:M122" headerRowCount="1">
-  <autoFilter ref="A1:M122"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseStudies" displayName="CaseStudies" ref="A1:N122" headerRowCount="1">
+  <autoFilter ref="A1:N122"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Category"/>
     <tableColumn id="3" name="Group"/>
@@ -216,6 +216,7 @@
     <tableColumn id="11" name="Formats"/>
     <tableColumn id="12" name="Tracked in git"/>
     <tableColumn id="13" name="Notes"/>
+    <tableColumn id="14" name="Prep pack (relative to Case_Study_Groups/)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
@@ -510,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1042,6 +1043,28 @@
       </c>
       <c r="B52" s="2">
         <f>B50+B51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Cases with a prep pack linked (Case Studies, Prep pack column)</t>
+        </is>
+      </c>
+      <c r="B53" s="2">
+        <f>COUNTA('Case Studies'!$N:$N)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Standalone cases with a pack in Case_Study_Groups/Standalone/</t>
+        </is>
+      </c>
+      <c r="B54" s="2">
+        <f>COUNTIF('Case Studies'!$N:$N,"Standalone/*")</f>
         <v/>
       </c>
     </row>
@@ -1935,7 +1958,11 @@
       </c>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Standalone/ — one folder per case (#67/#68/#69 share one pack); exact path in the Case Studies tab, Prep pack column</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2815,7 +2842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2831,6 +2858,7 @@
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="62" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2899,6 +2927,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Prep pack (relative to Case_Study_Groups/)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="n">
@@ -2960,6 +2993,11 @@
           <t>REST vs function calling vs MCP vs agent frameworks as layers; tool registry at scale; identity propagation</t>
         </is>
       </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -3021,6 +3059,11 @@
           <t>RAG vs tool calling; when a planner is justified; three memory layers; human approval; model routing</t>
         </is>
       </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -3082,6 +3125,11 @@
           <t>Context engineering as a funnel; cache first; model routing by task; decomposed latency budget</t>
         </is>
       </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>G09_Enterprise_Coding_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -3143,6 +3191,11 @@
           <t>Structured extraction as the seam; explainable ranking; AI judge that does not decide; fairness as a control</t>
         </is>
       </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/04_Recruiting_Platform/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -3204,6 +3257,11 @@
           <t>Clarifying questions; streaming + batch unified; Policy Gate; shared control plane, regional data planes</t>
         </is>
       </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>G17_Logistics_Exception_Handling.md</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -3261,6 +3319,11 @@
           <t>Minute-by-minute performance script. Built in Handbook Module 04</t>
         </is>
       </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -3318,6 +3381,11 @@
           <t>Minute-by-minute performance script. Built in Handbook Module 08 doc 3</t>
         </is>
       </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -3375,6 +3443,11 @@
           <t>Minute-by-minute performance script. Built in Handbook Module 05</t>
         </is>
       </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>G15_Agent_Platform_For_Non_Technical_Users.md</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -3432,6 +3505,11 @@
           <t>Minute-by-minute performance script. Built in Handbook Module 10</t>
         </is>
       </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>G12_Scoping_To_Deployed_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -3489,6 +3567,11 @@
           <t>Worked Design One. Ch 23 (system design patterns) is the vocabulary it uses.</t>
         </is>
       </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>G11_Deep_Research_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -3546,6 +3629,11 @@
           <t>Worked Design Two.</t>
         </is>
       </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>G04_SRE_Incident_Response_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -3599,6 +3687,11 @@
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>G11_Deep_Research_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -3652,6 +3745,11 @@
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr"/>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>G06_NL_Over_Governed_Data.md</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -3713,6 +3811,11 @@
           <t>Foundations-level worked example.</t>
         </is>
       </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/14_Travel_Agent_Worked_Example/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -3778,6 +3881,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -3843,6 +3951,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -3908,6 +4021,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>G06_NL_Over_Governed_Data.md</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -3973,6 +4091,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -4038,6 +4161,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/19_Air_Gapped_AI_System/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -4103,6 +4231,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>G13_Evaluation_And_Release_Gating.md</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -4168,6 +4301,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>G10_High_Volume_Batch_Pipeline.md</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -4233,6 +4371,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -4298,6 +4441,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/23_Reliable_Workflow_Orchestration/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
@@ -4363,6 +4511,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -4428,6 +4581,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/25_Configurable_Platform_Customer_Workflows/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -4493,6 +4651,11 @@
           <t>Source: The Forward Deployed Engineer System Design Interview (Kindle). Ch 21 V1 also has an uncondensed tutorial.</t>
         </is>
       </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/26_Enterprise_Chatbot_Platform/  [copied source files (folder)]</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -4558,6 +4721,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx. Has a short + full mock interview (01_internal_knowledge_assistant).</t>
         </is>
       </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
@@ -4623,6 +4791,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>G05_Sales_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -4688,6 +4861,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx. Has a short + full mock interview (03_financial_red_team (red-team variant)).</t>
         </is>
       </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
@@ -4753,6 +4931,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -4818,6 +5001,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -4883,6 +5071,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx. Has a short + full mock interview (04_sre_triage).</t>
         </is>
       </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>G04_SRE_Incident_Response_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -4948,6 +5141,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx. Has a short + full mock interview (05_multi_tenant_saas).</t>
         </is>
       </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -5013,6 +5211,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>G06_NL_Over_Governed_Data.md</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -5078,6 +5281,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -5143,6 +5351,11 @@
           <t>Answer keys also as docx (untracked) and in the canonical combined docx.</t>
         </is>
       </c>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>G06_NL_Over_Governed_Data.md</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -5204,6 +5417,11 @@
           <t>Only mock not drawn from a Module 01 worksheet. The other 4 mocks are listed against their worksheet rows.</t>
         </is>
       </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -5265,6 +5483,11 @@
           <t>§16 Case 1. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
@@ -5326,6 +5549,11 @@
           <t>§16 Case 2. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -5387,6 +5615,11 @@
           <t>§16 Case 3. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>G05_Sales_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
@@ -5448,6 +5681,11 @@
           <t>§16 Case 4. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -5509,6 +5747,11 @@
           <t>§16 Case 5. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N43" s="6" t="inlineStr">
+        <is>
+          <t>G10_High_Volume_Batch_Pipeline.md</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
@@ -5570,6 +5813,11 @@
           <t>§16 Case 6. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>G16_Real_Time_Call_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -5631,6 +5879,11 @@
           <t>§16 Case 7. Format: prompt / ask / weak vs strong answer / architecture / trade-offs / metrics / recommendation.</t>
         </is>
       </c>
+      <c r="N45" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -5692,6 +5945,11 @@
           <t>Question 1. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -5753,6 +6011,11 @@
           <t>Question 2. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N47" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
@@ -5814,6 +6077,11 @@
           <t>Question 3. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
@@ -5875,6 +6143,11 @@
           <t>Question 4. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>G05_Sales_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
@@ -5936,6 +6209,11 @@
           <t>Question 5. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>G10_High_Volume_Batch_Pipeline.md</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
@@ -5997,6 +6275,11 @@
           <t>Question 6. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
@@ -6058,6 +6341,11 @@
           <t>Question 7. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>G09_Enterprise_Coding_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
@@ -6119,6 +6407,11 @@
           <t>Question 8. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>G13_Evaluation_And_Release_Gating.md</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
@@ -6180,6 +6473,11 @@
           <t>Question 9. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N54" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
@@ -6241,6 +6539,11 @@
           <t>Question 10. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N55" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
@@ -6302,6 +6605,11 @@
           <t>Question 11. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>G13_Evaluation_And_Release_Gating.md</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
@@ -6363,6 +6671,11 @@
           <t>Question 12. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
@@ -6424,6 +6737,11 @@
           <t>Question 13. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N58" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
@@ -6485,6 +6803,11 @@
           <t>Question 14. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N59" s="6" t="inlineStr">
+        <is>
+          <t>G04_SRE_Incident_Response_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -6546,6 +6869,11 @@
           <t>Question 15. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>G16_Real_Time_Call_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
@@ -6607,6 +6935,11 @@
           <t>Question 16. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/60_Prioritize_AI_Use_Cases/60_Prioritize_AI_Use_Cases.md</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
@@ -6668,6 +7001,11 @@
           <t>Question 17. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N62" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/61_Scale_Prototype_To_Production/61_Scale_Prototype_To_Production.md</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
@@ -6729,6 +7067,11 @@
           <t>Question 18. Talking points + likely follow-up, not a full worked design.</t>
         </is>
       </c>
+      <c r="N63" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/62_Build_When_Customer_Data_Is_Poor/62_Build_When_Customer_Data_Is_Poor.md</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
@@ -6790,6 +7133,11 @@
           <t>One company threaded through the whole module; also told as a STAR story.</t>
         </is>
       </c>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
@@ -6847,6 +7195,11 @@
         </is>
       </c>
       <c r="M65" s="6" t="inlineStr"/>
+      <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>G15_Agent_Platform_For_Non_Technical_Users.md</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
@@ -6904,6 +7257,11 @@
         </is>
       </c>
       <c r="M66" s="6" t="inlineStr"/>
+      <c r="N66" s="6" t="inlineStr">
+        <is>
+          <t>G12_Scoping_To_Deployed_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
@@ -6965,6 +7323,11 @@
           <t>Tier 1 prompt 1 · reported at OpenAI FDE · tests: multi-system data unification, stakeholder surface area, evaluation as first-class. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>G17_Logistics_Exception_Handling.md</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
@@ -7026,6 +7389,11 @@
           <t>Tier 1 prompt 2 · reported at Decomposition classic · tests: mission clarification (response time vs cost vs equity), input mapping, sequencing by risk. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
@@ -7087,6 +7455,11 @@
           <t>Tier 1 prompt 3 · reported at Decomposition classic · tests: data-quality realism, phased scoping, regulatory constraints. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
@@ -7148,6 +7521,11 @@
           <t>Tier 1 prompt 4 · reported at Decomposition classic · tests: high-stakes HITL design, safety-first decomposition. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
@@ -7209,6 +7587,11 @@
           <t>Tier 1 prompt 5 · reported at OpenAI perf · tests: latency budget decomposition across retrieval, generation and network. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
@@ -7270,6 +7653,11 @@
           <t>Tier 1 prompt 6 · reported at OpenAI · tests: consumer-scale chat service design. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N72" s="6" t="inlineStr">
+        <is>
+          <t>G19_Consumer_Scale_Chat_Service.md</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
@@ -7331,6 +7719,11 @@
           <t>Tier 1 prompt 7 · reported at OpenAI · tests: enterprise search design. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N73" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
@@ -7392,6 +7785,11 @@
           <t>Tier 1 prompt 8 · reported at OpenAI · tests: training infrastructure under constraints. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>G20_Model_Development_And_Post_Training.md</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
@@ -7453,6 +7851,11 @@
           <t>Tier 1 prompt 9 · reported at OpenAI favorite · tests: full-stack inference latency reasoning. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>G21_LLM_Inference_Serving.md</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
@@ -7514,6 +7917,11 @@
           <t>Tier 1 prompt 10 · reported at Anthropic · tests: batching, queuing, synchronous waiting. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>G21_LLM_Inference_Serving.md</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
@@ -7575,6 +7983,11 @@
           <t>Tier 1 prompt 11 · reported at Anthropic · tests: distributed-systems fundamentals: capacity discovery, failover. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N77" s="6" t="inlineStr">
+        <is>
+          <t>G21_LLM_Inference_Serving.md</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
@@ -7636,6 +8049,11 @@
           <t>Tier 1 prompt 12 · reported at Anthropic · tests: throughput, load balancing, backpressure. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N78" s="6" t="inlineStr">
+        <is>
+          <t>G21_LLM_Inference_Serving.md</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n">
@@ -7697,6 +8115,11 @@
           <t>Tier 1 prompt 13 · reported at Anthropic · tests: chat service architecture at scale. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N79" s="6" t="inlineStr">
+        <is>
+          <t>G19_Consumer_Scale_Chat_Service.md</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="n">
@@ -7758,6 +8181,11 @@
           <t>Tier 1 prompt 14 · reported at Anthropic review · tests: design critique of batching/queuing. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N80" s="6" t="inlineStr">
+        <is>
+          <t>G21_LLM_Inference_Serving.md</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
@@ -7819,6 +8247,11 @@
           <t>Tier 1 prompt 15 · reported at Anthropic MLE · tests: agent learning and adaptation. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/80_Self_Adapting_Agent/80_Self_Adapting_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
@@ -7880,6 +8313,11 @@
           <t>Tier 1 prompt 16 · reported at Anthropic · tests: alignment / post-training trade-off. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N82" s="6" t="inlineStr">
+        <is>
+          <t>G20_Model_Development_And_Post_Training.md</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
@@ -7941,6 +8379,11 @@
           <t>Tier 1 prompt 17 · reported at Salesforce · tests: agent architecture end to end. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
@@ -8002,6 +8445,11 @@
           <t>Tier 1 prompt 18 · reported at Google · tests: on-device model constraints + alignment. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N84" s="6" t="inlineStr">
+        <is>
+          <t>G20_Model_Development_And_Post_Training.md</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
@@ -8063,6 +8511,11 @@
           <t>Tier 1 prompt 19 · reported at Cohere · tests: model development pipeline. Pattern: business goal first, data second, model last.</t>
         </is>
       </c>
+      <c r="N85" s="6" t="inlineStr">
+        <is>
+          <t>G20_Model_Development_And_Post_Training.md</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="n">
@@ -8124,6 +8577,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N86" s="6" t="inlineStr">
+        <is>
+          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n">
@@ -8185,6 +8643,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N87" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
@@ -8246,6 +8709,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N88" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
@@ -8307,6 +8775,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N89" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="n">
@@ -8368,6 +8841,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n">
@@ -8429,6 +8907,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N91" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
@@ -8490,6 +8973,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N92" s="6" t="inlineStr">
+        <is>
+          <t>G13_Evaluation_And_Release_Gating.md</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n">
@@ -8551,6 +9039,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>G08_Document_Review_Copilot.md</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="n">
@@ -8612,6 +9105,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N94" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n">
@@ -8673,6 +9171,11 @@
           <t>Debugging case, not a design case: answer with detect → contain → root-cause → prevent, on the design of the group's anchor.</t>
         </is>
       </c>
+      <c r="N95" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n">
@@ -8734,6 +9237,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N96" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n">
@@ -8795,6 +9303,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N97" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="n">
@@ -8856,6 +9369,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N98" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n">
@@ -8917,6 +9435,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/98_Personal_Assistant_With_Memory/98_Personal_Assistant_With_Memory.md</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="n">
@@ -8978,6 +9501,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N100" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n">
@@ -9039,6 +9567,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N101" s="6" t="inlineStr">
+        <is>
+          <t>Standalone/100_Production_LLM_Gateway/100_Production_LLM_Gateway.md</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="n">
@@ -9100,6 +9633,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N102" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n">
@@ -9161,6 +9699,11 @@
           <t>section 6 (Mock system design). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N103" s="6" t="inlineStr">
+        <is>
+          <t>G02_Customer_Support_Automation.md</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n">
@@ -9222,6 +9765,11 @@
           <t>section 7 (Design a research system). Framework-flavoured (LangChain/LangGraph) treatment of the same system; use it to add implementation detail to the anchor, not as a separate case.</t>
         </is>
       </c>
+      <c r="N104" s="6" t="inlineStr">
+        <is>
+          <t>G11_Deep_Research_Agent.md</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n">
@@ -9283,6 +9831,11 @@
           <t>§15 scenario 1. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N105" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="n">
@@ -9344,6 +9897,11 @@
           <t>§15 scenario 2. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N106" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n">
@@ -9405,6 +9963,11 @@
           <t>§15 scenario 3. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N107" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="n">
@@ -9466,6 +10029,11 @@
           <t>§15 scenario 4. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N108" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="n">
@@ -9527,6 +10095,11 @@
           <t>§15 scenario 5. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N109" s="6" t="inlineStr">
+        <is>
+          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="n">
@@ -9588,6 +10161,11 @@
           <t>§15 scenario 6. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N110" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="6" t="n">
@@ -9649,6 +10227,11 @@
           <t>§15 scenario 7. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N111" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="n">
@@ -9710,6 +10293,11 @@
           <t>§15 scenario 8. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N112" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="6" t="n">
@@ -9771,6 +10359,11 @@
           <t>§15 scenario 9. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N113" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="n">
@@ -9832,6 +10425,11 @@
           <t>§15 scenario 10. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N114" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="n">
@@ -9893,6 +10491,11 @@
           <t>§15 scenario 11. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N115" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="n">
@@ -9954,6 +10557,11 @@
           <t>§15 scenario 12. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N116" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="n">
@@ -10015,6 +10623,11 @@
           <t>§15 scenario 13. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N117" s="6" t="inlineStr">
+        <is>
+          <t>G10_High_Volume_Batch_Pipeline.md</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="n">
@@ -10076,6 +10689,11 @@
           <t>§15 scenario 14. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N118" s="6" t="inlineStr">
+        <is>
+          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="n">
@@ -10137,6 +10755,11 @@
           <t>§15 scenario 15. Shape: symptom / ask / causes / metrics / debug / now / later / prevent / say. Same 8 drivers as the drills.</t>
         </is>
       </c>
+      <c r="N119" s="6" t="inlineStr">
+        <is>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="n">
@@ -10194,6 +10817,11 @@
           <t>Section E: a scenario the interviewer may add that §15 does not cover; one 'senior answer' row.</t>
         </is>
       </c>
+      <c r="N120" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="n">
@@ -10251,6 +10879,11 @@
           <t>Section E: a scenario the interviewer may add that §15 does not cover; one 'senior answer' row.</t>
         </is>
       </c>
+      <c r="N121" s="6" t="inlineStr">
+        <is>
+          <t>G13_Evaluation_And_Release_Gating.md</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="6" t="n">
@@ -10306,6 +10939,11 @@
       <c r="M122" s="6" t="inlineStr">
         <is>
           <t>Section E: a scenario the interviewer may add that §15 does not cover; one 'senior answer' row.</t>
+        </is>
+      </c>
+      <c r="N122" s="6" t="inlineStr">
+        <is>
+          <t>G14_Observability_And_Production_Diagnosis.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new case study documents for G18, G19, and G20, covering consumer-scale chat service design, model development and post-training, and LLM inference serving strategies. Update G01 and G02 guides with improved question formatting for clarity and decision-making.
</commit_message>
<xml_diff>
--- a/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
+++ b/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>G04_SRE_Incident_Response_Agent.md</t>
+          <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>G05_Sales_Copilot.md</t>
+          <t>G05_Sales_Copilot/</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>G06_NL_Over_Governed_Data.md</t>
+          <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+          <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>G09_Enterprise_Coding_Assistant.md</t>
+          <t>G09_Enterprise_Coding_Assistant/</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>G10_High_Volume_Batch_Pipeline.md</t>
+          <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>G11_Deep_Research_Agent.md</t>
+          <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>G12_Scoping_To_Deployed_Agent.md</t>
+          <t>G12_Scoping_To_Deployed_Agent/</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
           <t>#53 Latency Regression in an LLM Application — Latency-regression drill. Anchor's percentile/path decomposition covers it.
 #54 RAG System with Poor Answer Quality — RAG-quality debugging drill. Delta: separate retrieval vs generation metrics; 5 minutes.
 #44 Incident: LLM costs exploded after launch — Cost-explosion incident. Delta: cost telemetry + kill switch; 5 minutes.
-#74 Diagnose high latency in an LLM inference pipeline — Reported OpenAI prompt: diagnose inference-pipeline latency at the serving layer (tokenization, network, batch size, KV cache, post-processing). Delta: the layer below the app. Also grouped conceptually with G21; prepare the stack walk once.
+#74 Diagnose high latency in an LLM inference pipeline — Reported OpenAI prompt: diagnose inference-pipeline latency at the serving layer (tokenization, network, batch size, KV cache, post-processing). Delta: the layer below the app. Also grouped conceptually with G20; prepare the stack walk once.
 #87 Latency spike after reranker and model-routing change — Incident: latency spike after reranker and routing change. Trace the path, compare before/after by stage, roll back the change.
 #88 Cost spike from prompt-template and cache-key regression — Incident: cost spike from a prompt-template and cache-key regression. Cost attribution by prompt version; cache key must include the version.
 #104 LLM cost increased 5× after rollout — §15 scenario 1: cost up 5× after rollout. Break spend by tenant/feature/model/prompt version; cap output, pause batch, route down.
@@ -1703,7 +1703,7 @@
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>G15_Agent_Platform_For_Non_Technical_Users.md</t>
+          <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>G19 Consumer-scale chat service</t>
+          <t>G18 Consumer-scale chat service</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -1811,14 +1811,14 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>G19_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>G20 Model development and post-training</t>
+          <t>G19 Model development and post-training</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -1849,14 +1849,14 @@
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>G20_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -1888,7 +1888,7 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>G16_Real_Time_Call_Assistant.md</t>
+          <t>G16_Real_Time_Call_Assistant/</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>G09_Enterprise_Coding_Assistant.md</t>
+          <t>G09_Enterprise_Coding_Assistant/</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>G15_Agent_Platform_For_Non_Technical_Users.md</t>
+          <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>G12_Scoping_To_Deployed_Agent.md</t>
+          <t>G12_Scoping_To_Deployed_Agent/</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>G11_Deep_Research_Agent.md</t>
+          <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>G04_SRE_Incident_Response_Agent.md</t>
+          <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       <c r="M13" s="6" t="inlineStr"/>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>G11_Deep_Research_Agent.md</t>
+          <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
       <c r="M14" s="6" t="inlineStr"/>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>G06_NL_Over_Governed_Data.md</t>
+          <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+          <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>G06_NL_Over_Governed_Data.md</t>
+          <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>G10_High_Volume_Batch_Pipeline.md</t>
+          <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>G05_Sales_Copilot.md</t>
+          <t>G05_Sales_Copilot/</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4863,7 @@
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>G04_SRE_Incident_Response_Agent.md</t>
+          <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>G06_NL_Over_Governed_Data.md</t>
+          <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>G06_NL_Over_Governed_Data.md</t>
+          <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="N41" s="6" t="inlineStr">
         <is>
-          <t>G05_Sales_Copilot.md</t>
+          <t>G05_Sales_Copilot/</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+          <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>G10_High_Volume_Batch_Pipeline.md</t>
+          <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
     </row>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>G16_Real_Time_Call_Assistant.md</t>
+          <t>G16_Real_Time_Call_Assistant/</t>
         </is>
       </c>
     </row>
@@ -5881,7 +5881,7 @@
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -6013,7 +6013,7 @@
       </c>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="N48" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="N49" s="6" t="inlineStr">
         <is>
-          <t>G05_Sales_Copilot.md</t>
+          <t>G05_Sales_Copilot/</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="N50" s="6" t="inlineStr">
         <is>
-          <t>G10_High_Volume_Batch_Pipeline.md</t>
+          <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="N51" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>G09_Enterprise_Coding_Assistant.md</t>
+          <t>G09_Enterprise_Coding_Assistant/</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6409,7 @@
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -6541,7 +6541,7 @@
       </c>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6673,7 @@
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -6739,7 +6739,7 @@
       </c>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6805,7 @@
       </c>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>G04_SRE_Incident_Response_Agent.md</t>
+          <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>G16_Real_Time_Call_Assistant.md</t>
+          <t>G16_Real_Time_Call_Assistant/</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7135,7 @@
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -7197,7 +7197,7 @@
       <c r="M65" s="6" t="inlineStr"/>
       <c r="N65" s="6" t="inlineStr">
         <is>
-          <t>G15_Agent_Platform_For_Non_Technical_Users.md</t>
+          <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       <c r="M66" s="6" t="inlineStr"/>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>G12_Scoping_To_Deployed_Agent.md</t>
+          <t>G12_Scoping_To_Deployed_Agent/</t>
         </is>
       </c>
     </row>
@@ -7589,7 +7589,7 @@
       </c>
       <c r="N71" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -7604,7 +7604,7 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>G19 Consumer-scale chat service</t>
+          <t>G18 Consumer-scale chat service</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>G19_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service.md</t>
         </is>
       </c>
     </row>
@@ -7721,7 +7721,7 @@
       </c>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -7736,7 +7736,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>G20 Model development and post-training</t>
+          <t>G19 Model development and post-training</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>G20_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training.md</t>
         </is>
       </c>
     </row>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="N76" s="6" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="N77" s="6" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>G19 Consumer-scale chat service</t>
+          <t>G18 Consumer-scale chat service</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>G19_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service.md</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8132,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>G21 LLM inference serving infrastructure</t>
+          <t>G20 LLM inference serving infrastructure</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>G21_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving.md</t>
         </is>
       </c>
     </row>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>G20 Model development and post-training</t>
+          <t>G19 Model development and post-training</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>G20_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training.md</t>
         </is>
       </c>
     </row>
@@ -8381,7 +8381,7 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -8396,7 +8396,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>G20 Model development and post-training</t>
+          <t>G19 Model development and post-training</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>G20_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training.md</t>
         </is>
       </c>
     </row>
@@ -8462,7 +8462,7 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>G20 Model development and post-training</t>
+          <t>G19 Model development and post-training</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="N85" s="6" t="inlineStr">
         <is>
-          <t>G20_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training.md</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8579,7 @@
       </c>
       <c r="N86" s="6" t="inlineStr">
         <is>
-          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+          <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
     </row>
@@ -8645,7 +8645,7 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="N88" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -8777,7 +8777,7 @@
       </c>
       <c r="N89" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -8843,7 +8843,7 @@
       </c>
       <c r="N90" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="N91" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="N92" s="6" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="N93" s="6" t="inlineStr">
         <is>
-          <t>G08_Document_Review_Copilot.md</t>
+          <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="N94" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -9173,7 +9173,7 @@
       </c>
       <c r="N95" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9239,7 @@
       </c>
       <c r="N96" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9305,7 +9305,7 @@
       </c>
       <c r="N97" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9371,7 +9371,7 @@
       </c>
       <c r="N98" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9503,7 +9503,7 @@
       </c>
       <c r="N100" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9635,7 @@
       </c>
       <c r="N102" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9701,7 +9701,7 @@
       </c>
       <c r="N103" s="6" t="inlineStr">
         <is>
-          <t>G02_Customer_Support_Automation.md</t>
+          <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
       </c>
       <c r="N104" s="6" t="inlineStr">
         <is>
-          <t>G11_Deep_Research_Agent.md</t>
+          <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="N105" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -9899,7 +9899,7 @@
       </c>
       <c r="N106" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="N107" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -10031,7 +10031,7 @@
       </c>
       <c r="N108" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -10097,7 +10097,7 @@
       </c>
       <c r="N109" s="6" t="inlineStr">
         <is>
-          <t>G07_Secure_Multi_Tenant_AI_Platform.md</t>
+          <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
     </row>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="N110" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10229,7 @@
       </c>
       <c r="N111" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10295,7 +10295,7 @@
       </c>
       <c r="N112" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -10361,7 +10361,7 @@
       </c>
       <c r="N113" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="N114" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="N115" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10559,7 +10559,7 @@
       </c>
       <c r="N116" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10625,7 +10625,7 @@
       </c>
       <c r="N117" s="6" t="inlineStr">
         <is>
-          <t>G10_High_Volume_Batch_Pipeline.md</t>
+          <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
     </row>
@@ -10691,7 +10691,7 @@
       </c>
       <c r="N118" s="6" t="inlineStr">
         <is>
-          <t>G01_Enterprise_Knowledge_Assistant.md</t>
+          <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
     </row>
@@ -10757,7 +10757,7 @@
       </c>
       <c r="N119" s="6" t="inlineStr">
         <is>
-          <t>G03_Tool_Using_Agent_With_Safety_Controls.md</t>
+          <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
     </row>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="N120" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>
@@ -10881,7 +10881,7 @@
       </c>
       <c r="N121" s="6" t="inlineStr">
         <is>
-          <t>G13_Evaluation_And_Release_Gating.md</t>
+          <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
     </row>
@@ -10943,7 +10943,7 @@
       </c>
       <c r="N122" s="6" t="inlineStr">
         <is>
-          <t>G14_Observability_And_Production_Diagnosis.md</t>
+          <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new resources for AI Engineer interview preparation, including an updated CASE_STUDY_INDEX.xlsx, a new Agent Evaluation Playbook Sketchnote, and two new PDF documents on system architecture and agent design. Additionally, enhance the Recruiting Platform handbook with improved table formatting and a new self-adapting agent interview template for better clarity and usability.
</commit_message>
<xml_diff>
--- a/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
+++ b/06_Interview_Prep/CASE_STUDY_INDEX.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -99,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +127,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -200,9 +212,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseStudies" displayName="CaseStudies" ref="A1:N122" headerRowCount="1">
-  <autoFilter ref="A1:N122"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseStudies" displayName="CaseStudies" ref="A1:O122" headerRowCount="1">
+  <autoFilter ref="A1:O122"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Category"/>
     <tableColumn id="3" name="Group"/>
@@ -217,6 +229,7 @@
     <tableColumn id="12" name="Tracked in git"/>
     <tableColumn id="13" name="Notes"/>
     <tableColumn id="14" name="Prep pack (relative to Case_Study_Groups/)"/>
+    <tableColumn id="15" name="Site page (Forward Deployed)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
@@ -511,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1078,17 @@
       </c>
       <c r="B54" s="2">
         <f>COUNTIF('Case Studies'!$N:$N,"Standalone/*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Cases with a live site page (Case Studies, Site page column)</t>
+        </is>
+      </c>
+      <c r="B55" s="2">
+        <f>COUNTIF('Case Studies'!$O:$O,"https://*")</f>
         <v/>
       </c>
     </row>
@@ -1082,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1117,7 @@
     <col width="80" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1134,6 +1159,11 @@
       <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Day-before pack (Case_Study_Groups/)</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Site page (Forward Deployed)</t>
         </is>
       </c>
     </row>
@@ -1191,6 +1221,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1238,6 +1273,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1279,6 +1319,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1316,6 +1361,11 @@
           <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sre-incident-response-agent</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1351,6 +1401,11 @@
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>G05_Sales_Copilot/</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sales-copilot</t>
         </is>
       </c>
     </row>
@@ -1391,6 +1446,11 @@
           <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/nl-over-governed-data</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1427,6 +1487,11 @@
       <c r="H8" s="4" t="inlineStr">
         <is>
           <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/secure-multi-tenant-ai-platform</t>
         </is>
       </c>
     </row>
@@ -1470,6 +1535,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1504,6 +1574,11 @@
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>G09_Enterprise_Coding_Assistant/</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/enterprise-coding-assistant</t>
         </is>
       </c>
     </row>
@@ -1544,6 +1619,11 @@
           <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/high-volume-batch-pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1581,6 +1661,11 @@
           <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/deep-research-agent</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1615,6 +1700,11 @@
       <c r="H13" s="4" t="inlineStr">
         <is>
           <t>G12_Scoping_To_Deployed_Agent/</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/scoping-to-deployed-agent</t>
         </is>
       </c>
     </row>
@@ -1654,6 +1744,11 @@
       <c r="H14" s="4" t="inlineStr">
         <is>
           <t>G13_Evaluation_And_Release_Gating/</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
         </is>
       </c>
     </row>
@@ -1706,6 +1801,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1742,6 +1842,11 @@
           <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/agent-platform-for-non-technical-users</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1775,7 +1880,12 @@
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>G17_Logistics_Exception_Handling.md</t>
+          <t>G17_Logistics_Exception_Handling/</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/logistics-exception-handling</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1921,12 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>G18_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service/</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/consumer-scale-chat-service</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1964,12 @@
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>G19_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training/</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/model-development/model-development-and-post-training</t>
         </is>
       </c>
     </row>
@@ -1888,7 +2008,12 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -1925,6 +2050,11 @@
       <c r="H21" s="4" t="inlineStr">
         <is>
           <t>G16_Real_Time_Call_Assistant/</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/real-time-call-assistant</t>
         </is>
       </c>
     </row>
@@ -1963,8 +2093,36 @@
           <t>Standalone/ — one folder per case (#67/#68/#69 share one pack); exact path in the Case Studies tab, Prep pack column</t>
         </is>
       </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId21"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2842,7 +3000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N122"/>
+  <dimension ref="A1:O122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2859,6 +3017,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="62" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2932,6 +3091,11 @@
           <t>Prep pack (relative to Case_Study_Groups/)</t>
         </is>
       </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Site page (Forward Deployed)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="n">
@@ -2998,6 +3162,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O2" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -3064,6 +3233,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O3" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -3130,6 +3304,11 @@
           <t>G09_Enterprise_Coding_Assistant/</t>
         </is>
       </c>
+      <c r="O4" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/enterprise-coding-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -3196,6 +3375,11 @@
           <t>Standalone/04_Recruiting_Platform/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O5" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/recruiting-platform</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -3259,7 +3443,12 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>G17_Logistics_Exception_Handling.md</t>
+          <t>G17_Logistics_Exception_Handling/</t>
+        </is>
+      </c>
+      <c r="O6" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/logistics-exception-handling</t>
         </is>
       </c>
     </row>
@@ -3324,6 +3513,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -3386,6 +3580,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O8" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -3448,6 +3647,11 @@
           <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/agent-platform-for-non-technical-users</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -3510,6 +3714,11 @@
           <t>G12_Scoping_To_Deployed_Agent/</t>
         </is>
       </c>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/scoping-to-deployed-agent</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -3572,6 +3781,11 @@
           <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/deep-research-agent</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -3634,6 +3848,11 @@
           <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sre-incident-response-agent</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -3692,6 +3911,11 @@
           <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/deep-research-agent</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -3750,6 +3974,11 @@
           <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
+      <c r="O14" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/nl-over-governed-data</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -3816,6 +4045,11 @@
           <t>Standalone/14_Travel_Agent_Worked_Example/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/travel-agent-worked-example</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -3886,6 +4120,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O16" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -3956,6 +4195,11 @@
           <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/secure-multi-tenant-ai-platform</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -4026,6 +4270,11 @@
           <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
+      <c r="O18" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/nl-over-governed-data</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -4096,6 +4345,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O19" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -4166,6 +4420,11 @@
           <t>Standalone/19_Air_Gapped_AI_System/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O20" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/air-gapped-ai-system</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -4236,6 +4495,11 @@
           <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
+      <c r="O21" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -4306,6 +4570,11 @@
           <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
+      <c r="O22" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/high-volume-batch-pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -4376,6 +4645,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O23" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -4446,6 +4720,11 @@
           <t>Standalone/23_Reliable_Workflow_Orchestration/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/reliable-workflow-orchestration</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
@@ -4516,6 +4795,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -4586,6 +4870,11 @@
           <t>Standalone/25_Configurable_Platform_Customer_Workflows/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O26" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/configurable-platform-customer-workflows</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -4656,6 +4945,11 @@
           <t>Standalone/26_Enterprise_Chatbot_Platform/  [copied source files (folder)]</t>
         </is>
       </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/enterprise-chatbot-platform</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -4726,6 +5020,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
@@ -4796,6 +5095,11 @@
           <t>G05_Sales_Copilot/</t>
         </is>
       </c>
+      <c r="O29" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sales-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -4866,6 +5170,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O30" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
@@ -4936,6 +5245,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O31" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -5006,6 +5320,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O32" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -5076,6 +5395,11 @@
           <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
+      <c r="O33" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sre-incident-response-agent</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -5146,6 +5470,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O34" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -5216,6 +5545,11 @@
           <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
+      <c r="O35" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/nl-over-governed-data</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -5286,6 +5620,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O36" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -5356,6 +5695,11 @@
           <t>G06_NL_Over_Governed_Data/</t>
         </is>
       </c>
+      <c r="O37" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/nl-over-governed-data</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -5422,6 +5766,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O38" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -5488,6 +5837,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O39" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
@@ -5554,6 +5908,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O40" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -5620,6 +5979,11 @@
           <t>G05_Sales_Copilot/</t>
         </is>
       </c>
+      <c r="O41" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sales-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
@@ -5686,6 +6050,11 @@
           <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
+      <c r="O42" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/secure-multi-tenant-ai-platform</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -5752,6 +6121,11 @@
           <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
+      <c r="O43" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/high-volume-batch-pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
@@ -5818,6 +6192,11 @@
           <t>G16_Real_Time_Call_Assistant/</t>
         </is>
       </c>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/real-time-call-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -5884,6 +6263,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O45" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -5950,6 +6334,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O46" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -6016,6 +6405,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O47" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
@@ -6082,6 +6476,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O48" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
@@ -6148,6 +6547,11 @@
           <t>G05_Sales_Copilot/</t>
         </is>
       </c>
+      <c r="O49" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sales-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
@@ -6214,6 +6618,11 @@
           <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
+      <c r="O50" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/high-volume-batch-pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
@@ -6280,6 +6689,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O51" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
@@ -6346,6 +6760,11 @@
           <t>G09_Enterprise_Coding_Assistant/</t>
         </is>
       </c>
+      <c r="O52" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/enterprise-coding-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
@@ -6412,6 +6831,11 @@
           <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
+      <c r="O53" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
@@ -6478,6 +6902,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O54" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
@@ -6544,6 +6973,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O55" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
@@ -6610,6 +7044,11 @@
           <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
+      <c r="O56" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
@@ -6676,6 +7115,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O57" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
@@ -6742,6 +7186,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O58" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
@@ -6808,6 +7257,11 @@
           <t>G04_SRE_Incident_Response_Agent/</t>
         </is>
       </c>
+      <c r="O59" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/sre-incident-response-agent</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -6874,6 +7328,11 @@
           <t>G16_Real_Time_Call_Assistant/</t>
         </is>
       </c>
+      <c r="O60" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/real-time-call-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
@@ -6940,6 +7399,11 @@
           <t>Standalone/60_Prioritize_AI_Use_Cases/60_Prioritize_AI_Use_Cases.md</t>
         </is>
       </c>
+      <c r="O61" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/prioritize-ai-use-cases</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
@@ -7006,6 +7470,11 @@
           <t>Standalone/61_Scale_Prototype_To_Production/61_Scale_Prototype_To_Production.md</t>
         </is>
       </c>
+      <c r="O62" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/scale-prototype-to-production</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
@@ -7072,6 +7541,11 @@
           <t>Standalone/62_Build_When_Customer_Data_Is_Poor/62_Build_When_Customer_Data_Is_Poor.md</t>
         </is>
       </c>
+      <c r="O63" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/build-when-customer-data-is-poor</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
@@ -7138,6 +7612,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O64" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
@@ -7200,6 +7679,11 @@
           <t>G15_Agent_Platform_For_Non_Technical_Users/</t>
         </is>
       </c>
+      <c r="O65" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/agent-platform-for-non-technical-users</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
@@ -7262,6 +7746,11 @@
           <t>G12_Scoping_To_Deployed_Agent/</t>
         </is>
       </c>
+      <c r="O66" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/scoping-to-deployed-agent</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
@@ -7325,7 +7814,12 @@
       </c>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>G17_Logistics_Exception_Handling.md</t>
+          <t>G17_Logistics_Exception_Handling/</t>
+        </is>
+      </c>
+      <c r="O67" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/logistics-exception-handling</t>
         </is>
       </c>
     </row>
@@ -7394,6 +7888,11 @@
           <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
         </is>
       </c>
+      <c r="O68" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/decomposition-classics-67-68-69</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
@@ -7460,6 +7959,11 @@
           <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
         </is>
       </c>
+      <c r="O69" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/decomposition-classics-67-68-69</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
@@ -7526,6 +8030,11 @@
           <t>Standalone/Decomposition_Classics_67_68_69/Decomposition_Classics_67_68_69.md</t>
         </is>
       </c>
+      <c r="O70" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/judgement-and-decomposition/decomposition-classics-67-68-69</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
@@ -7592,6 +8101,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O71" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
@@ -7655,7 +8169,12 @@
       </c>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>G18_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service/</t>
+        </is>
+      </c>
+      <c r="O72" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/consumer-scale-chat-service</t>
         </is>
       </c>
     </row>
@@ -7724,6 +8243,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O73" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
@@ -7787,7 +8311,12 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>G19_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training/</t>
+        </is>
+      </c>
+      <c r="O74" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/model-development/model-development-and-post-training</t>
         </is>
       </c>
     </row>
@@ -7853,7 +8382,12 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="O75" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -7919,7 +8453,12 @@
       </c>
       <c r="N76" s="6" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="O76" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -7985,7 +8524,12 @@
       </c>
       <c r="N77" s="6" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="O77" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8595,12 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="O78" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -8117,7 +8666,12 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>G18_Consumer_Scale_Chat_Service.md</t>
+          <t>G18_Consumer_Scale_Chat_Service/</t>
+        </is>
+      </c>
+      <c r="O79" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/consumer-scale-chat-service</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8737,12 @@
       </c>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>G20_LLM_Inference_Serving.md</t>
+          <t>G20_LLM_Inference_Serving/</t>
+        </is>
+      </c>
+      <c r="O80" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/llm-inference-serving</t>
         </is>
       </c>
     </row>
@@ -8252,6 +8811,11 @@
           <t>Standalone/80_Self_Adapting_Agent/80_Self_Adapting_Agent.md</t>
         </is>
       </c>
+      <c r="O81" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/self-adapting-agent</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
@@ -8315,7 +8879,12 @@
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>G19_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training/</t>
+        </is>
+      </c>
+      <c r="O82" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/model-development/model-development-and-post-training</t>
         </is>
       </c>
     </row>
@@ -8384,6 +8953,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O83" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
@@ -8447,7 +9021,12 @@
       </c>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>G19_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training/</t>
+        </is>
+      </c>
+      <c r="O84" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/model-development/model-development-and-post-training</t>
         </is>
       </c>
     </row>
@@ -8513,7 +9092,12 @@
       </c>
       <c r="N85" s="6" t="inlineStr">
         <is>
-          <t>G19_Model_Development_And_Post_Training.md</t>
+          <t>G19_Model_Development_And_Post_Training/</t>
+        </is>
+      </c>
+      <c r="O85" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/model-development/model-development-and-post-training</t>
         </is>
       </c>
     </row>
@@ -8582,6 +9166,11 @@
           <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
+      <c r="O86" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/secure-multi-tenant-ai-platform</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n">
@@ -8648,6 +9237,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O87" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
@@ -8714,6 +9308,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O88" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
@@ -8780,6 +9379,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O89" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="n">
@@ -8846,6 +9450,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O90" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n">
@@ -8912,6 +9521,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O91" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
@@ -8978,6 +9592,11 @@
           <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
+      <c r="O92" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n">
@@ -9044,6 +9663,11 @@
           <t>G08_Document_Review_Copilot/</t>
         </is>
       </c>
+      <c r="O93" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/document-review-copilot</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="n">
@@ -9110,6 +9734,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O94" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n">
@@ -9176,6 +9805,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O95" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n">
@@ -9242,6 +9876,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O96" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n">
@@ -9308,6 +9947,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O97" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="n">
@@ -9374,6 +10018,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O98" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n">
@@ -9440,6 +10089,11 @@
           <t>Standalone/98_Personal_Assistant_With_Memory/98_Personal_Assistant_With_Memory.md</t>
         </is>
       </c>
+      <c r="O99" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/personal-assistant-with-memory</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="n">
@@ -9506,6 +10160,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O100" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n">
@@ -9572,6 +10231,11 @@
           <t>Standalone/100_Production_LLM_Gateway/100_Production_LLM_Gateway.md</t>
         </is>
       </c>
+      <c r="O101" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/standalone-designs/production-llm-gateway</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="n">
@@ -9638,6 +10302,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O102" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n">
@@ -9704,6 +10373,11 @@
           <t>G02_Customer_Support_Automation/</t>
         </is>
       </c>
+      <c r="O103" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/customer-support-automation</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n">
@@ -9770,6 +10444,11 @@
           <t>G11_Deep_Research_Agent/</t>
         </is>
       </c>
+      <c r="O104" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/deep-research-agent</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n">
@@ -9836,6 +10515,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O105" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="n">
@@ -9902,6 +10586,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O106" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n">
@@ -9968,6 +10657,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O107" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="n">
@@ -10034,6 +10728,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O108" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="n">
@@ -10100,6 +10799,11 @@
           <t>G07_Secure_Multi_Tenant_AI_Platform/</t>
         </is>
       </c>
+      <c r="O109" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/secure-multi-tenant-ai-platform</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="n">
@@ -10166,6 +10870,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O110" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="6" t="n">
@@ -10232,6 +10941,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O111" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="n">
@@ -10298,6 +11012,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O112" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="6" t="n">
@@ -10364,6 +11083,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O113" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="n">
@@ -10430,6 +11154,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O114" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="n">
@@ -10496,6 +11225,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O115" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="n">
@@ -10562,6 +11296,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O116" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="n">
@@ -10628,6 +11367,11 @@
           <t>G10_High_Volume_Batch_Pipeline/</t>
         </is>
       </c>
+      <c r="O117" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/platforms-and-scale/high-volume-batch-pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="n">
@@ -10694,6 +11438,11 @@
           <t>G01_Enterprise_Knowledge_Assistant/</t>
         </is>
       </c>
+      <c r="O118" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/knowledge-retrieval/enterprise-knowledge-assistant</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="n">
@@ -10760,6 +11509,11 @@
           <t>G03_Tool_Using_Agent_With_Safety_Controls/</t>
         </is>
       </c>
+      <c r="O119" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/agents-that-act/tool-using-agent-with-safety-controls</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="n">
@@ -10822,6 +11576,11 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O120" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="n">
@@ -10884,6 +11643,11 @@
           <t>G13_Evaluation_And_Release_Gating/</t>
         </is>
       </c>
+      <c r="O121" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/evaluation-and-release-gating</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="6" t="n">
@@ -10946,11 +11710,139 @@
           <t>G14_Observability_And_Production_Diagnosis/</t>
         </is>
       </c>
+      <c r="O122" s="12" t="inlineStr">
+        <is>
+          <t>https://forward-deployed-sigma.vercel.app/modules/15-fde-case-studies/delivery-evaluation-operations/observability-and-production-diagnosis</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId121"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId122"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>